<commit_message>
level 3 NN model update and main function
</commit_message>
<xml_diff>
--- a/ASPECT_calibration_pipeline/level_3/datasets/ASPECT/REF_MEAS_upd_wl.xlsx
+++ b/ASPECT_calibration_pipeline/level_3/datasets/ASPECT/REF_MEAS_upd_wl.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valtterimj/Downloads/Työ/Aalto/Hera/Pipeline/Asteroid-spectra/v3.0/datasets/ASPECT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valtterimj/Downloads/Työ/Aalto/Hera/Pipeline/main/ASPECT_calibration_pipeline/level_3/datasets/ASPECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8FF8B8C-E107-AA40-AC88-94A65BBBA36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46DC1AF-1C98-A941-8226-CEA15CFF3497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12120" yWindow="660" windowWidth="16520" windowHeight="16040" activeTab="1" xr2:uid="{3B7B7263-57CE-4670-B472-5AB98268D44C}"/>
   </bookViews>
@@ -3240,7 +3240,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42333228-403B-7F4C-BA26-71F42800C60A}">
-  <dimension ref="A3:A43"/>
+  <dimension ref="A3:A42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
@@ -3369,67 +3369,62 @@
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31">
-        <v>1225</v>
+      <c r="A31" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>41</v>
+      <c r="A36">
+        <v>1400</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37">
-        <v>1400</v>
+      <c r="A37" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A43">
+      <c r="A42">
         <v>1575</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new NN trained for ASPECT vis-nir1-nir2 and nir1-nir2
</commit_message>
<xml_diff>
--- a/ASPECT_calibration_pipeline/level_3/datasets/ASPECT/REF_MEAS_upd_wl.xlsx
+++ b/ASPECT_calibration_pipeline/level_3/datasets/ASPECT/REF_MEAS_upd_wl.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/valtterimj/Downloads/Työ/Aalto/Hera/Pipeline/main/ASPECT_calibration_pipeline/level_3/datasets/ASPECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46DC1AF-1C98-A941-8226-CEA15CFF3497}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37B5C659-FA67-4848-951A-1100BC07C5C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12120" yWindow="660" windowWidth="16520" windowHeight="16040" activeTab="1" xr2:uid="{3B7B7263-57CE-4670-B472-5AB98268D44C}"/>
   </bookViews>

</xml_diff>